<commit_message>
email phone, website copy and edit option addded
</commit_message>
<xml_diff>
--- a/excel/Batch_03_Leads_Tracker.xlsx
+++ b/excel/Batch_03_Leads_Tracker.xlsx
@@ -528,10 +528,10 @@
 The redesign can be kept affordable, usually around $200 to $800 depending on what you need. You do not need to pay anything upfront. Payment is only after the website is delivered and you are happy with the result.</v>
       </c>
       <c r="L2" t="str">
-        <v>Draft</v>
+        <v>Sent</v>
       </c>
       <c r="M2" t="str">
-        <v/>
+        <v>2026-09-17</v>
       </c>
       <c r="N2" t="str">
         <v>Re: A simpler enquiry route for Capitol Carpets</v>
@@ -606,10 +606,10 @@
 The redesign can be kept affordable, usually around $200 to $800 depending on what you need. You do not need to pay anything upfront. Payment is only after the website is delivered and you are happy with the result.</v>
       </c>
       <c r="L3" t="str">
-        <v>Draft</v>
+        <v>Sent</v>
       </c>
       <c r="M3" t="str">
-        <v/>
+        <v>2026-09-17</v>
       </c>
       <c r="N3" t="str">
         <v>Re: Updating the first impression of London Electric Lighting</v>
@@ -686,10 +686,10 @@
 The redesign can be kept affordable, usually around $200 to $800 depending on what you need. You do not need to pay anything upfront. Payment is only after the website is delivered and you are happy with the result.</v>
       </c>
       <c r="L4" t="str">
-        <v>Draft</v>
+        <v>Sent</v>
       </c>
       <c r="M4" t="str">
-        <v/>
+        <v>2026-09-17</v>
       </c>
       <c r="N4" t="str">
         <v>Re: A few unfinished details on the Amazing Carpets website</v>
@@ -765,10 +765,10 @@
 The redesign can be kept affordable, usually around $200 to $800 depending on what you need. You do not need to pay anything upfront. Payment is only after the website is delivered and you are happy with the result.</v>
       </c>
       <c r="L5" t="str">
-        <v>Draft</v>
+        <v>Sent</v>
       </c>
       <c r="M5" t="str">
-        <v/>
+        <v>2026-09-17</v>
       </c>
       <c r="N5" t="str">
         <v>Re: An easier project enquiry for KAB Decorating</v>
@@ -843,10 +843,10 @@
 The redesign can be kept affordable, usually around $200 to $800 depending on what you need. You do not need to pay anything upfront. Payment is only after the website is delivered and you are happy with the result.</v>
       </c>
       <c r="L6" t="str">
-        <v>Draft</v>
+        <v>Sent</v>
       </c>
       <c r="M6" t="str">
-        <v/>
+        <v>2026-09-17</v>
       </c>
       <c r="N6" t="str">
         <v>Re: Making the 1-2-1 Plumbers homepage easier to use</v>
@@ -921,10 +921,10 @@
 The redesign can be kept affordable, usually around $200 to $800 depending on what you need. You do not need to pay anything upfront. Payment is only after the website is delivered and you are happy with the result.</v>
       </c>
       <c r="L7" t="str">
-        <v>Draft</v>
+        <v>Sent</v>
       </c>
       <c r="M7" t="str">
-        <v/>
+        <v>2026-09-17</v>
       </c>
       <c r="N7" t="str">
         <v>Re: A clearer service journey for Better Heating and Lighting</v>
@@ -1000,10 +1000,10 @@
 The redesign can be kept affordable, usually around $200 to $800 depending on what you need. You do not need to pay anything upfront. Payment is only after the website is delivered and you are happy with the result.</v>
       </c>
       <c r="L8" t="str">
-        <v>Draft</v>
+        <v>Sent</v>
       </c>
       <c r="M8" t="str">
-        <v/>
+        <v>2026-09-17</v>
       </c>
       <c r="N8" t="str">
         <v>Re: Making Advanced Clean easier to enquire with</v>
@@ -1158,10 +1158,10 @@
 The redesign can be kept affordable, usually around $200 to $800 depending on what you need. You do not need to pay anything upfront. Payment is only after the website is delivered and you are happy with the result.</v>
       </c>
       <c r="L10" t="str">
-        <v>Draft</v>
+        <v>Sent</v>
       </c>
       <c r="M10" t="str">
-        <v/>
+        <v>2026-09-17</v>
       </c>
       <c r="N10" t="str">
         <v>Re: A more visual home for John Lawler's craftsmanship</v>
@@ -1236,10 +1236,10 @@
 The redesign can be kept affordable, usually around $200 to $800 depending on what you need. You do not need to pay anything upfront. Payment is only after the website is delivered and you are happy with the result.</v>
       </c>
       <c r="L11" t="str">
-        <v>Draft</v>
+        <v>Sent</v>
       </c>
       <c r="M11" t="str">
-        <v/>
+        <v>2026-09-17</v>
       </c>
       <c r="N11" t="str">
         <v>Re: A clearer quotation path for Thomas Roofing</v>
@@ -1314,10 +1314,10 @@
 The redesign can be kept affordable, usually around $200 to $800 depending on what you need. You do not need to pay anything upfront. Payment is only after the website is delivered and you are happy with the result.</v>
       </c>
       <c r="L12" t="str">
-        <v>Draft</v>
+        <v>Sent</v>
       </c>
       <c r="M12" t="str">
-        <v/>
+        <v>2026-09-17</v>
       </c>
       <c r="N12" t="str">
         <v>Re: A more polished online experience for Elite Dry Cleaners</v>
@@ -1392,10 +1392,10 @@
 The redesign can be kept affordable, usually around $200 to $800 depending on what you need. You do not need to pay anything upfront. Payment is only after the website is delivered and you are happy with the result.</v>
       </c>
       <c r="L13" t="str">
-        <v>Draft</v>
+        <v>Sent</v>
       </c>
       <c r="M13" t="str">
-        <v/>
+        <v>2026-09-17</v>
       </c>
       <c r="N13" t="str">
         <v>Re: A faster MOT and service booking journey for New Generation Cars</v>
@@ -1470,10 +1470,10 @@
 The redesign can be kept affordable, usually around $200 to $800 depending on what you need. You do not need to pay anything upfront. Payment is only after the website is delivered and you are happy with the result.</v>
       </c>
       <c r="L14" t="str">
-        <v>Draft</v>
+        <v>Sent</v>
       </c>
       <c r="M14" t="str">
-        <v/>
+        <v>2026-09-17</v>
       </c>
       <c r="N14" t="str">
         <v>Re: Making Carpet4Life's flooring range easier to explore</v>
@@ -1548,10 +1548,10 @@
 The redesign can be kept affordable, usually around $200 to $800 depending on what you need. You do not need to pay anything upfront. Payment is only after the website is delivered and you are happy with the result.</v>
       </c>
       <c r="L15" t="str">
-        <v>Draft</v>
+        <v>Sent</v>
       </c>
       <c r="M15" t="str">
-        <v/>
+        <v>2026-09-17</v>
       </c>
       <c r="N15" t="str">
         <v>Re: A clearer service-led homepage for Absolute</v>
@@ -1606,10 +1606,10 @@
 Portfolio: ksnirob.com</v>
       </c>
       <c r="H16" t="str">
-        <v>Sent</v>
+        <v>Draft</v>
       </c>
       <c r="I16" t="str">
-        <v>2026-09-08</v>
+        <v/>
       </c>
       <c r="J16" t="str">
         <v>Re: Removing placeholder content from Wills Roofing's homepage</v>
@@ -1704,10 +1704,10 @@
 The redesign can be kept affordable, usually around $200 to $800 depending on what you need. You do not need to pay anything upfront. Payment is only after the website is delivered and you are happy with the result.</v>
       </c>
       <c r="L17" t="str">
-        <v>Draft</v>
+        <v>Sent</v>
       </c>
       <c r="M17" t="str">
-        <v/>
+        <v>2026-09-17</v>
       </c>
       <c r="N17" t="str">
         <v>Re: A cleaner emergency-glazing journey for LMC Glass</v>
@@ -1783,10 +1783,10 @@
 The redesign can be kept affordable, usually around $200 to $800 depending on what you need. You do not need to pay anything upfront. Payment is only after the website is delivered and you are happy with the result.</v>
       </c>
       <c r="L18" t="str">
-        <v>Draft</v>
+        <v>Sent</v>
       </c>
       <c r="M18" t="str">
-        <v/>
+        <v>2026-09-17</v>
       </c>
       <c r="N18" t="str">
         <v>Re: A more focused project showcase for David Banks &amp; Company</v>
@@ -1861,10 +1861,10 @@
 The redesign can be kept affordable, usually around $200 to $800 depending on what you need. You do not need to pay anything upfront. Payment is only after the website is delivered and you are happy with the result.</v>
       </c>
       <c r="L19" t="str">
-        <v>Draft</v>
+        <v>Sent</v>
       </c>
       <c r="M19" t="str">
-        <v/>
+        <v>2026-09-17</v>
       </c>
       <c r="N19" t="str">
         <v>Re: A more visual showcase for The Oakhill Workshop</v>
@@ -1943,10 +1943,10 @@
 The redesign can be kept affordable, usually around $200 to $800 depending on what you need. You do not need to pay anything upfront. Payment is only after the website is delivered and you are happy with the result.</v>
       </c>
       <c r="L20" t="str">
-        <v>Draft</v>
+        <v>Sent</v>
       </c>
       <c r="M20" t="str">
-        <v/>
+        <v>2026-09-17</v>
       </c>
       <c r="N20" t="str">
         <v>Re: Clarifying Haringey Glass &amp; Glazing's homepage message</v>
@@ -2022,10 +2022,10 @@
 The redesign can be kept affordable, usually around $200 to $800 depending on what you need. You do not need to pay anything upfront. Payment is only after the website is delivered and you are happy with the result.</v>
       </c>
       <c r="L21" t="str">
-        <v>Draft</v>
+        <v>Sent</v>
       </c>
       <c r="M21" t="str">
-        <v/>
+        <v>2026-09-17</v>
       </c>
       <c r="N21" t="str">
         <v>Re: Replacing the stale notice on Carpet Factory Outlet's homepage</v>
@@ -2055,7 +2055,7 @@
   </ignoredErrors>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="0" showErrorMessage="1" sqref="H2:H1000 L2:L1000 P2:P1000">
-      <formula1>"Draft,Sent,Replied,Closed"</formula1>
+      <formula1>"Draft,Sent,Replied,Mail Not Found,Bounce Back,Closed"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="R2:R1000">
       <formula1>"Win,Lost"</formula1>

</xml_diff>